<commit_message>
set new token update blacklist record
</commit_message>
<xml_diff>
--- a/data/evaluation/summary/Experiment.xlsx
+++ b/data/evaluation/summary/Experiment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github_ThisPC\muict_thai_legal_rag\data\evaluation\summary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373F03D7-01B1-449B-9BF5-F5581E90E4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DBF670-62EA-4577-A0B5-E14DE9DF6C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
   <si>
     <t>system</t>
   </si>
@@ -75,34 +75,67 @@
     <t>retrieval_top1</t>
   </si>
   <si>
-    <t>0.9235412474849095</t>
-  </si>
-  <si>
-    <t>0.8148893360160966</t>
-  </si>
-  <si>
-    <t>0.8628820542301427</t>
-  </si>
-  <si>
-    <t>0.7488493230444941</t>
-  </si>
-  <si>
-    <t>3.0333780257600047</t>
-  </si>
-  <si>
     <t>retrieval_topn</t>
   </si>
   <si>
-    <t>0.9255533199195171</t>
-  </si>
-  <si>
-    <t>0.8209255533199196</t>
-  </si>
-  <si>
-    <t>0.7524671840567213</t>
-  </si>
-  <si>
     <t>Top-k</t>
+  </si>
+  <si>
+    <t>0.9221311475409836</t>
+  </si>
+  <si>
+    <t>0.8135245901639344</t>
+  </si>
+  <si>
+    <t>0.7476327463520086</t>
+  </si>
+  <si>
+    <t>3.0079935889392444</t>
+  </si>
+  <si>
+    <t>0.9241803278688525</t>
+  </si>
+  <si>
+    <t>0.8661592505854802</t>
+  </si>
+  <si>
+    <t>0.7513173302107728</t>
+  </si>
+  <si>
+    <t>3.0500423336033253</t>
+  </si>
+  <si>
+    <t>graph</t>
+  </si>
+  <si>
+    <t>0.8831967213114754</t>
+  </si>
+  <si>
+    <t>0.7684426229508197</t>
+  </si>
+  <si>
+    <t>0.8200445615404632</t>
+  </si>
+  <si>
+    <t>0.1408744659256954</t>
+  </si>
+  <si>
+    <t>0.1351709140131271</t>
+  </si>
+  <si>
+    <t>2828.9221311475408</t>
+  </si>
+  <si>
+    <t>181.29918032786884</t>
+  </si>
+  <si>
+    <t>0.1715420635281604</t>
+  </si>
+  <si>
+    <t>4.742863936271981</t>
+  </si>
+  <si>
+    <t>4.914405999800141</t>
   </si>
 </sst>
 </file>
@@ -421,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -485,7 +518,7 @@
         <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -493,19 +526,19 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>497</v>
+        <v>488</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="E2">
+        <v>0.86103629976580798</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -513,6 +546,9 @@
       <c r="H2">
         <v>0</v>
       </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
       <c r="J2">
         <v>0</v>
       </c>
@@ -523,13 +559,13 @@
         <v>0</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N2">
         <v>0</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P2">
         <v>3</v>
@@ -537,19 +573,19 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B3">
-        <v>497</v>
+        <v>488</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3">
+        <v>0.81967213114754101</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="E3">
-        <v>0.86724154450512603</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>24</v>
@@ -560,6 +596,9 @@
       <c r="H3">
         <v>0</v>
       </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
       <c r="J3">
         <v>0</v>
       </c>
@@ -569,16 +608,66 @@
       <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3">
-        <v>3.0732561529139</v>
+      <c r="M3" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
-      <c r="O3">
-        <v>3.0732561529139</v>
+      <c r="O3" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="P3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4">
+        <v>488</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4">
+        <v>0.68307962529274002</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4">
+        <v>0.895587441007622</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4">
+        <v>3010.2213114754099</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4">
         <v>3</v>
       </c>
     </row>

</xml_diff>